<commit_message>
Test Report hinzugefügt, Status nachgetragen, Logfiles verlinkt Stories_Req_Design_Test_G1.xlsx bereit zum finalen Review
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_G1.xlsx
+++ b/doc/Stories_Req_Design_Test_G1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E02FA11-2AFA-46F3-A04C-D951203DD1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24820C61-226B-4030-BF65-4820F1BCA3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="191">
   <si>
     <t>User Story ID</t>
   </si>
@@ -492,9 +492,6 @@
   </si>
   <si>
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
-  </si>
-  <si>
-    <t>US_G1_1\3</t>
   </si>
   <si>
     <t>System ist nach max. 60 Sekunden einsatzbereit und liest analoge Audiosignale über die Klinke-Schnittstelle ein</t>
@@ -534,6 +531,90 @@
   <si>
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät 
 </t>
+  </si>
+  <si>
+    <t>David Rösch</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>Traceability zu allen Anforderungen</t>
+  </si>
+  <si>
+    <t>Versionsverwaltung:</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Template übernommen und für Projekt aktualisiert</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>User Stories begonnen</t>
+  </si>
+  <si>
+    <t>2.1</t>
+  </si>
+  <si>
+    <t>User Stories fertig, Anforderungen begonnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anforderungen nach Review überabeitet </t>
+  </si>
+  <si>
+    <t>3.0</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>2.2</t>
+  </si>
+  <si>
+    <t>User Stories und Anforderungen final reviewed, Test Cases Formulierung begonnen</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>Status von User Stories, Anforderungen und Test Cases aktualisiert</t>
+  </si>
+  <si>
+    <t>Was wurde gemacht:</t>
+  </si>
+  <si>
+    <t>Test-Cases formuliert, zusätzlich Test-Umgebung beschrieben</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>Design-Kriterien hinzugefügt</t>
+  </si>
+  <si>
+    <t>Test-Cases finalisiert und allgemeine Dokument Fehler behoben</t>
+  </si>
+  <si>
+    <t>3.4</t>
+  </si>
+  <si>
+    <t>Test-Cases final reviewed</t>
+  </si>
+  <si>
+    <t>test_protokolle\TC_G1_1_signed.pdf</t>
+  </si>
+  <si>
+    <t>test_protokolle\TC_G1_2_signed.pdf</t>
+  </si>
+  <si>
+    <t>test_protokolle\TC_G1_3_signed.pdf</t>
+  </si>
+  <si>
+    <t>test_protokolle\TC_G1_4_signed.pdf</t>
   </si>
   <si>
     <r>
@@ -636,82 +717,60 @@
       <t xml:space="preserve"> (BPM, Tonart,...) zu ermitteln.
 Am Einspielgerät kann die Geschwindigkeit des aktuellen Musikstücks verändert werden. Die Veränderung wird live angezeigt und ausgegeben</t>
     </r>
-  </si>
-  <si>
-    <t>David Rösch</t>
-  </si>
-  <si>
-    <t>3.2</t>
-  </si>
-  <si>
-    <t>US_G1_1\2\3\5</t>
-  </si>
-  <si>
-    <t>Traceability zu allen Anforderungen</t>
-  </si>
-  <si>
-    <t>Versionsverwaltung:</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>Template übernommen und für Projekt aktualisiert</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>User Stories begonnen</t>
-  </si>
-  <si>
-    <t>2.1</t>
-  </si>
-  <si>
-    <t>User Stories fertig, Anforderungen begonnen</t>
-  </si>
-  <si>
-    <t>User Stories nach review überarbeitet, Anforderungen fertig gestellt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anforderungen nach Review überabeitet </t>
-  </si>
-  <si>
-    <t>3.0</t>
-  </si>
-  <si>
-    <t>3.1</t>
-  </si>
-  <si>
-    <t>2.2</t>
-  </si>
-  <si>
-    <t>2.3</t>
-  </si>
-  <si>
-    <t>Test-Cases fertig formuliert, zusätzlich Test-Umgebung beschrieben</t>
-  </si>
-  <si>
-    <t>User Stories und Anforderungen final reviewed, Test Cases Formulierung begonnen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-Cases final reviewed </t>
-  </si>
-  <si>
-    <t>4.0</t>
-  </si>
-  <si>
-    <t>Status von User Stories, Anforderungen und Test Cases aktualisiert</t>
-  </si>
-  <si>
-    <t>Was wurde gemacht:</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Begleitend zur Durchführung der Tests wurden Protokolle sowie eine Test-Zusammenfassung begelegt. Die Protokolle sind als Log verlinkt und die Zusammenfassung liegt unter folgendem Link:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>test_protokolle\Test_Report_G1_14062026.pdf</t>
+  </si>
+  <si>
+    <t>US_G1_1
+US_G1_2
+US_G1_3
+US_G1_5</t>
+  </si>
+  <si>
+    <t>US_G1_1
+US_G1_3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -795,6 +854,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -816,7 +883,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -881,26 +948,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -988,10 +1035,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1029,10 +1077,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1081,6 +1129,35 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1093,61 +1170,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1427,182 +1479,207 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A1" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="51"/>
-    </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="C1" s="41"/>
+    </row>
+    <row r="2" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A2" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="53"/>
-    </row>
-    <row r="3" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="C2" s="43"/>
+    </row>
+    <row r="3" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A3" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="53"/>
-    </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="C3" s="43"/>
+    </row>
+    <row r="4" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A4" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="52" t="s">
-        <v>161</v>
-      </c>
-      <c r="C4" s="53"/>
-    </row>
-    <row r="5" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="B4" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="C4" s="43"/>
+    </row>
+    <row r="5" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A5" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="54" t="s">
-        <v>181</v>
-      </c>
-      <c r="C5" s="55"/>
-    </row>
-    <row r="6" spans="1:3" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.7">
+      <c r="B5" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" s="45"/>
+    </row>
+    <row r="6" spans="1:3" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="56">
-        <v>46183</v>
-      </c>
-      <c r="C6" s="57"/>
-    </row>
-    <row r="8" spans="1:3" ht="21" x14ac:dyDescent="0.4">
-      <c r="A8" s="46" t="s">
+      <c r="B6" s="46">
+        <v>46188</v>
+      </c>
+      <c r="C6" s="47"/>
+    </row>
+    <row r="8" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+      <c r="A8" s="35" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>176</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="C9" s="55">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="B8" s="61" t="s">
-        <v>183</v>
-      </c>
-      <c r="C8" s="61" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="58" t="s">
+      <c r="B10" s="38" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="59" t="s">
+      <c r="C10" s="55">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="39" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="59" t="s">
+      <c r="B11" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="B10" s="59" t="s">
+      <c r="C11" s="55">
+        <v>46136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="39" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="60" t="s">
+      <c r="C12" s="55">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B13" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="C13" s="55">
+        <v>46140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="60" t="s">
-        <v>176</v>
-      </c>
-      <c r="B12" s="59" t="s">
-        <v>172</v>
-      </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="60" t="s">
+      <c r="B14" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="55">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B13" s="59" t="s">
-        <v>173</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="59" t="s">
+      <c r="C15" s="55">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="55">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="38" t="s">
+        <v>182</v>
+      </c>
+      <c r="C17" s="55">
+        <v>46182</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="39" t="s">
         <v>174</v>
       </c>
-      <c r="B14" s="59" t="s">
-        <v>179</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="60" t="s">
+      <c r="B18" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="B15" s="59" t="s">
-        <v>178</v>
-      </c>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="60" t="s">
-        <v>162</v>
-      </c>
-      <c r="B16" s="59" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="60" t="s">
-        <v>181</v>
-      </c>
-      <c r="B17" s="59" t="s">
-        <v>182</v>
-      </c>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="49"/>
-      <c r="B18" s="47"/>
-    </row>
-    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="49"/>
-      <c r="B19" s="47"/>
-    </row>
-    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="49"/>
-      <c r="B20" s="47"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="48"/>
-      <c r="B21" s="48"/>
+      <c r="C18" s="55">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="37"/>
+      <c r="B19" s="36"/>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="37"/>
+      <c r="B20" s="36"/>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="37"/>
+      <c r="B21" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1612,18 +1689,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.44140625" style="27" customWidth="1"/>
-    <col min="4" max="4" width="36.109375" style="27" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" style="27" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="27" customWidth="1"/>
     <col min="5" max="6" width="24" style="9" customWidth="1"/>
-    <col min="7" max="7" width="25.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.44140625" style="6"/>
+    <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1646,7 +1723,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>113</v>
       </c>
@@ -1660,16 +1737,16 @@
         <v>120</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>114</v>
       </c>
@@ -1683,16 +1760,16 @@
         <v>118</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>115</v>
       </c>
@@ -1706,16 +1783,16 @@
         <v>119</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>116</v>
       </c>
@@ -1729,16 +1806,16 @@
         <v>109</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>117</v>
       </c>
@@ -1752,16 +1829,16 @@
         <v>111</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D11" s="26"/>
     </row>
   </sheetData>
@@ -1797,20 +1874,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.44140625" style="27" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="24" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" style="6"/>
-    <col min="5" max="5" width="13.33203125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" style="6"/>
-    <col min="7" max="8" width="23.44140625" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.33203125" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.44140625" style="6"/>
+    <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" style="27" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="24" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="6"/>
+    <col min="7" max="7" width="23.42578125" style="26" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>17</v>
       </c>
@@ -1829,7 +1907,7 @@
       <c r="F1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="60" t="s">
         <v>10</v>
       </c>
       <c r="H1" s="21" t="s">
@@ -1839,7 +1917,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>122</v>
       </c>
@@ -1858,15 +1936,15 @@
       <c r="F2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>163</v>
+      <c r="G2" s="25" t="s">
+        <v>189</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>123</v>
       </c>
@@ -1885,7 +1963,7 @@
       <c r="F3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="25" t="s">
         <v>114</v>
       </c>
       <c r="H3" s="7"/>
@@ -1893,7 +1971,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>125</v>
       </c>
@@ -1912,15 +1990,15 @@
       <c r="F4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>163</v>
+      <c r="G4" s="25" t="s">
+        <v>189</v>
       </c>
       <c r="H4" s="7"/>
       <c r="I4" s="7" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>126</v>
       </c>
@@ -1939,7 +2017,7 @@
       <c r="F5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="25" t="s">
         <v>114</v>
       </c>
       <c r="H5" s="7"/>
@@ -1947,7 +2025,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>127</v>
       </c>
@@ -1966,7 +2044,7 @@
       <c r="F6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="25" t="s">
         <v>115</v>
       </c>
       <c r="H6" s="7"/>
@@ -1974,7 +2052,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>128</v>
       </c>
@@ -1993,15 +2071,15 @@
       <c r="F7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>163</v>
+      <c r="G7" s="25" t="s">
+        <v>189</v>
       </c>
       <c r="H7" s="7"/>
       <c r="I7" s="7" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>124</v>
       </c>
@@ -2020,15 +2098,15 @@
       <c r="F8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>150</v>
+      <c r="G8" s="25" t="s">
+        <v>190</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="7" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>129</v>
       </c>
@@ -2047,7 +2125,7 @@
       <c r="F9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="25" t="s">
         <v>116</v>
       </c>
       <c r="H9" s="7"/>
@@ -2055,7 +2133,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>130</v>
       </c>
@@ -2074,7 +2152,7 @@
       <c r="F10" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="25" t="s">
         <v>117</v>
       </c>
       <c r="H10" s="7"/>
@@ -2145,25 +2223,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.44140625" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" customWidth="1"/>
-    <col min="4" max="4" width="25.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="C1" s="35" t="s">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="C1" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C2" s="39" t="s">
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C2" s="52" t="s">
         <v>62</v>
       </c>
       <c r="D2" s="13" t="s">
@@ -2176,8 +2254,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="40"/>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="53"/>
       <c r="D3" s="14" t="s">
         <v>139</v>
       </c>
@@ -2188,7 +2266,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="10"/>
       <c r="C4" s="2" t="s">
         <v>74</v>
@@ -2203,7 +2281,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
         <v>59</v>
       </c>
@@ -2220,7 +2298,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
@@ -2235,7 +2313,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2" t="s">
         <v>57</v>
@@ -2250,7 +2328,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="10"/>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -2265,7 +2343,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="10"/>
       <c r="C9" s="12" t="s">
         <v>138</v>
@@ -2280,7 +2358,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>65</v>
       </c>
@@ -2290,90 +2368,90 @@
       <c r="C11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="36" t="s">
+      <c r="D11" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="37"/>
-      <c r="F11" s="38"/>
-    </row>
-    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E12" s="56"/>
+      <c r="F12" s="56"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
         <v>68</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D13" s="56"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="56"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>69</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>70</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="43"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
         <v>72</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="43"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="43"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2390,18 +2468,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.77734375" style="30" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" style="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -2424,10 +2502,10 @@
         <v>23</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="26" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="26" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>143</v>
       </c>
@@ -2435,23 +2513,25 @@
         <v>147</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="25"/>
+        <v>87</v>
+      </c>
+      <c r="F2" s="57" t="s">
+        <v>183</v>
+      </c>
       <c r="G2" s="25" t="s">
         <v>122</v>
       </c>
       <c r="H2" s="25" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="26" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>144</v>
       </c>
@@ -2462,20 +2542,22 @@
         <v>149</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="25"/>
+        <v>87</v>
+      </c>
+      <c r="F3" s="57" t="s">
+        <v>184</v>
+      </c>
       <c r="G3" s="25" t="s">
         <v>123</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="26" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="26" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>145</v>
       </c>
@@ -2483,15 +2565,17 @@
         <v>148</v>
       </c>
       <c r="C4" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="D4" s="25" t="s">
-        <v>153</v>
-      </c>
       <c r="E4" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="25"/>
+        <v>87</v>
+      </c>
+      <c r="F4" s="57" t="s">
+        <v>185</v>
+      </c>
       <c r="G4" s="25" t="s">
         <v>125</v>
       </c>
@@ -2499,7 +2583,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="26" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>146</v>
       </c>
@@ -2507,15 +2591,17 @@
         <v>147</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="25"/>
+        <v>88</v>
+      </c>
+      <c r="F5" s="57" t="s">
+        <v>186</v>
+      </c>
       <c r="G5" s="25" t="s">
         <v>124</v>
       </c>
@@ -2523,7 +2609,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6"/>
       <c r="B6"/>
       <c r="C6"/>
@@ -2533,145 +2619,155 @@
       <c r="G6"/>
       <c r="H6" s="27"/>
     </row>
-    <row r="7" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7"/>
-      <c r="B7" s="45" t="s">
-        <v>160</v>
-      </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
+      <c r="B7" s="54" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="54"/>
       <c r="H7" s="27"/>
     </row>
-    <row r="8" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
       <c r="H8" s="27"/>
     </row>
-    <row r="9" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
       <c r="H9" s="27"/>
     </row>
-    <row r="10" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
       <c r="H10" s="27"/>
     </row>
-    <row r="11" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
       <c r="H11" s="27"/>
     </row>
-    <row r="12" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="54"/>
+      <c r="G12" s="54"/>
       <c r="H12" s="27"/>
     </row>
-    <row r="13" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="54"/>
       <c r="H13" s="27"/>
     </row>
-    <row r="14" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
       <c r="H14" s="27"/>
     </row>
-    <row r="15" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
-      <c r="B15" s="44"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
       <c r="H15" s="27"/>
     </row>
-    <row r="16" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
-      <c r="B16"/>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16" s="9"/>
-      <c r="F16"/>
-      <c r="G16"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
       <c r="H16" s="27"/>
     </row>
-    <row r="17" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
-      <c r="B17"/>
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17" s="9"/>
-      <c r="F17"/>
-      <c r="G17"/>
+      <c r="B17" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
       <c r="H17" s="30"/>
     </row>
-    <row r="18" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
-      <c r="B18"/>
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18" s="9"/>
-      <c r="F18"/>
-      <c r="G18"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="58"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58"/>
       <c r="H18" s="30"/>
     </row>
-    <row r="19" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19"/>
-      <c r="B19"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19" s="9"/>
-      <c r="F19"/>
-      <c r="G19"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58"/>
       <c r="H19" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B7:G15"/>
+  <mergeCells count="2">
+    <mergeCell ref="B7:G16"/>
+    <mergeCell ref="B17:G17"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{62012F5C-BAC2-4E5A-B276-7672ECAA27AB}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{395DD683-3C7B-45C8-9763-3297FE0B0F1E}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{FDA3A799-002E-45BD-969B-CC45A1134BB8}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{6BFA7090-54E3-437D-B3D9-683A350FF2B6}"/>
+    <hyperlink ref="B17:G17" r:id="rId5" display="test_protokolle\Test_Report_G1_14062026.pdf" xr:uid="{B584271E-61FC-44A6-ABF9-044D7CD6DAEB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -2696,17 +2792,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.109375" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -2726,7 +2822,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
@@ -2746,7 +2842,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -2766,7 +2862,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -2786,7 +2882,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>29</v>
       </c>
@@ -2797,7 +2893,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -2808,7 +2904,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2817,7 +2913,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2826,7 +2922,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -2835,7 +2931,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2844,7 +2940,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2853,7 +2949,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2862,7 +2958,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2871,7 +2967,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2880,7 +2976,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2889,7 +2985,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2898,7 +2994,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -2907,7 +3003,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -2916,7 +3012,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2925,7 +3021,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>

</xml_diff>

<commit_message>
Stories_Req_Design_Test_G1.xlsx final aktualisiert Architektur Nachverfolgung nachgetragen
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_G1.xlsx
+++ b/doc/Stories_Req_Design_Test_G1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24820C61-226B-4030-BF65-4820F1BCA3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4D0C23-6807-4131-8D12-2BC6A662E208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="190">
   <si>
     <t>User Story ID</t>
   </si>
@@ -191,27 +191,6 @@
   </si>
   <si>
     <t>ArchEl_12</t>
-  </si>
-  <si>
-    <t>ArchEl_13</t>
-  </si>
-  <si>
-    <t>ArchEl_14</t>
-  </si>
-  <si>
-    <t>ArchEl_15</t>
-  </si>
-  <si>
-    <t>ArchEl_16</t>
-  </si>
-  <si>
-    <t>ArchEl_17</t>
-  </si>
-  <si>
-    <t>ArchEl_18</t>
-  </si>
-  <si>
-    <t>ArchEl_19</t>
   </si>
   <si>
     <t>Aufwand</t>
@@ -765,6 +744,33 @@
     <t>US_G1_1
 US_G1_3</t>
   </si>
+  <si>
+    <t>ArchEl_1 
+ArchEl_2 
+ArchEl_7
+ArchEl_8</t>
+  </si>
+  <si>
+    <t>ArchEl_5
+ArchEl_10</t>
+  </si>
+  <si>
+    <t>ArchEl_2
+ArchEl_3
+ArchEl_4
+ArchEl_12</t>
+  </si>
+  <si>
+    <t>ArchEl_3
+ArchEl_4
+ArchEL_9</t>
+  </si>
+  <si>
+    <t>4.1</t>
+  </si>
+  <si>
+    <t>Architektur Nachverfolgung nachgetragen</t>
+  </si>
 </sst>
 </file>
 
@@ -883,7 +889,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1034,12 +1040,83 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1134,6 +1211,27 @@
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1152,12 +1250,6 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1176,26 +1268,47 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1487,182 +1600,189 @@
   <sheetData>
     <row r="1" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A1" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B1" s="40" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="41"/>
+        <v>82</v>
+      </c>
+      <c r="B1" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="48"/>
     </row>
     <row r="2" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A2" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="43"/>
+        <v>87</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="50"/>
     </row>
     <row r="3" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A3" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="C3" s="43"/>
+        <v>88</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="50"/>
     </row>
     <row r="4" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A4" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="C4" s="43"/>
+        <v>83</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="50"/>
     </row>
     <row r="5" spans="1:3" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A5" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="44" t="s">
-        <v>174</v>
-      </c>
-      <c r="C5" s="45"/>
+        <v>85</v>
+      </c>
+      <c r="B5" s="51" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="52"/>
     </row>
     <row r="6" spans="1:3" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" s="46">
-        <v>46188</v>
-      </c>
-      <c r="C6" s="47"/>
+        <v>84</v>
+      </c>
+      <c r="B6" s="45">
+        <v>46189</v>
+      </c>
+      <c r="C6" s="46"/>
     </row>
     <row r="8" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A8" s="35" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="C9" s="55">
+        <v>157</v>
+      </c>
+      <c r="C9" s="40">
         <v>46133</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="C10" s="55">
+        <v>159</v>
+      </c>
+      <c r="C10" s="40">
         <v>46133</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="C11" s="55">
+        <v>161</v>
+      </c>
+      <c r="C11" s="40">
         <v>46136</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="C12" s="55">
+        <v>162</v>
+      </c>
+      <c r="C12" s="40">
         <v>46139</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="C13" s="55">
+        <v>166</v>
+      </c>
+      <c r="C13" s="40">
         <v>46140</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="C14" s="55">
+        <v>172</v>
+      </c>
+      <c r="C14" s="40">
         <v>46147</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="C15" s="55">
+        <v>170</v>
+      </c>
+      <c r="C15" s="40">
         <v>46148</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="55">
+        <v>173</v>
+      </c>
+      <c r="C16" s="40">
         <v>46163</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>182</v>
-      </c>
-      <c r="C17" s="55">
+        <v>175</v>
+      </c>
+      <c r="C17" s="40">
         <v>46182</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="55">
+        <v>168</v>
+      </c>
+      <c r="C18" s="40">
         <v>46188</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="37"/>
-      <c r="B19" s="36"/>
+      <c r="A19" s="39" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="C19" s="40">
+        <v>46189</v>
+      </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="37"/>
@@ -1725,16 +1845,16 @@
     </row>
     <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" s="34" t="s">
         <v>113</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>120</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>31</v>
@@ -1743,21 +1863,21 @@
         <v>33</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>31</v>
@@ -1766,21 +1886,21 @@
         <v>33</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>31</v>
@@ -1789,21 +1909,21 @@
         <v>33</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B5" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="34" t="s">
-        <v>108</v>
-      </c>
       <c r="D5" s="34" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="E5" s="19" t="s">
         <v>31</v>
@@ -1812,21 +1932,21 @@
         <v>33</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D6" s="34" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>31</v>
@@ -1835,7 +1955,7 @@
         <v>33</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1879,12 +1999,12 @@
     <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.42578125" style="27" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" style="24" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="4" max="4" width="12.28515625" style="6" customWidth="1"/>
     <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="6"/>
     <col min="7" max="7" width="23.42578125" style="26" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="63" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="26" customWidth="1"/>
     <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
@@ -1907,25 +2027,25 @@
       <c r="F1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="60" t="s">
+      <c r="G1" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="44" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>31</v>
@@ -1937,22 +2057,24 @@
         <v>33</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="H2" s="41" t="s">
+        <v>184</v>
+      </c>
+      <c r="I2" s="60" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>31</v>
@@ -1964,22 +2086,24 @@
         <v>33</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7" t="s">
-        <v>144</v>
+        <v>107</v>
+      </c>
+      <c r="H3" s="41" t="s">
+        <v>186</v>
+      </c>
+      <c r="I3" s="60" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>125</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>132</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>31</v>
@@ -1991,22 +2115,24 @@
         <v>33</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7" t="s">
-        <v>145</v>
+        <v>182</v>
+      </c>
+      <c r="H4" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="60" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>31</v>
@@ -2018,22 +2144,24 @@
         <v>33</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+      <c r="H5" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" s="60" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>31</v>
@@ -2045,22 +2173,24 @@
         <v>33</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7" t="s">
-        <v>144</v>
+        <v>108</v>
+      </c>
+      <c r="H6" s="41" t="s">
+        <v>187</v>
+      </c>
+      <c r="I6" s="60" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>31</v>
@@ -2072,22 +2202,24 @@
         <v>33</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7" t="s">
-        <v>144</v>
+        <v>182</v>
+      </c>
+      <c r="H7" s="41" t="s">
+        <v>185</v>
+      </c>
+      <c r="I7" s="60" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>31</v>
@@ -2099,22 +2231,24 @@
         <v>33</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>190</v>
-      </c>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7" t="s">
-        <v>146</v>
+        <v>183</v>
+      </c>
+      <c r="H8" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="60" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="31" t="s">
-        <v>136</v>
-      </c>
       <c r="C9" s="23" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>31</v>
@@ -2126,22 +2260,24 @@
         <v>33</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7" t="s">
-        <v>143</v>
+        <v>109</v>
+      </c>
+      <c r="H9" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="60" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>31</v>
@@ -2153,11 +2289,13 @@
         <v>33</v>
       </c>
       <c r="G10" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7" t="s">
-        <v>143</v>
+        <v>110</v>
+      </c>
+      <c r="H10" s="62" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" s="60" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2171,12 +2309,6 @@
             <xm:f>LookUp!$A$2:$A$6</xm:f>
           </x14:formula1>
           <xm:sqref>C11:C18</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
-          <x14:formula1>
-            <xm:f>LookUp!$E$2:$E$20</xm:f>
-          </x14:formula1>
-          <xm:sqref>H2:H19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
           <x14:formula1>
@@ -2214,6 +2346,12 @@
           </x14:formula1>
           <xm:sqref>I2:I10</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
+          <x14:formula1>
+            <xm:f>LookUp!$E$2:$E$13</xm:f>
+          </x14:formula1>
+          <xm:sqref>H11:H19</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -2233,225 +2371,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="C1" s="48" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="C1" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C2" s="52" t="s">
-        <v>62</v>
+      <c r="C2" s="57" t="s">
+        <v>55</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="53"/>
+      <c r="C3" s="58"/>
       <c r="D3" s="14" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="10"/>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="19" t="s">
-        <v>68</v>
-      </c>
       <c r="E6" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="10"/>
       <c r="C8" s="2" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="10"/>
       <c r="C9" s="12" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="50"/>
-      <c r="F11" s="51"/>
+        <v>72</v>
+      </c>
+      <c r="D11" s="54" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="55"/>
+      <c r="F11" s="56"/>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D12" s="56" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" s="56"/>
-      <c r="F12" s="56"/>
+        <v>73</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D13" s="56"/>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
+        <v>75</v>
+      </c>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D15" s="56"/>
-      <c r="E15" s="56"/>
-      <c r="F15" s="56"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
+        <v>74</v>
+      </c>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
+        <v>68</v>
+      </c>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2502,111 +2640,111 @@
         <v>23</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="26" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D2" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="E2" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="42" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="H2" s="25" t="s">
         <v>147</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="E2" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="57" t="s">
-        <v>183</v>
-      </c>
-      <c r="G2" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="57" t="s">
-        <v>184</v>
+        <v>80</v>
+      </c>
+      <c r="F3" s="42" t="s">
+        <v>177</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="26" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="D4" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>152</v>
-      </c>
       <c r="E4" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="57" t="s">
-        <v>185</v>
+        <v>80</v>
+      </c>
+      <c r="F4" s="42" t="s">
+        <v>178</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="57" t="s">
-        <v>186</v>
+        <v>81</v>
+      </c>
+      <c r="F5" s="42" t="s">
+        <v>179</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="H5" s="25" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
@@ -2621,136 +2759,136 @@
     </row>
     <row r="7" spans="1:8" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7"/>
-      <c r="B7" s="54" t="s">
-        <v>187</v>
-      </c>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
+      <c r="B7" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="66"/>
       <c r="H7" s="27"/>
     </row>
     <row r="8" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="69"/>
       <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
+      <c r="B9" s="67"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="G9" s="69"/>
       <c r="H9" s="27"/>
     </row>
     <row r="10" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="68"/>
+      <c r="G10" s="69"/>
       <c r="H10" s="27"/>
     </row>
     <row r="11" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
+      <c r="E11" s="68"/>
+      <c r="F11" s="68"/>
+      <c r="G11" s="69"/>
       <c r="H11" s="27"/>
     </row>
     <row r="12" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
+      <c r="B12" s="67"/>
+      <c r="C12" s="68"/>
+      <c r="D12" s="68"/>
+      <c r="E12" s="68"/>
+      <c r="F12" s="68"/>
+      <c r="G12" s="69"/>
       <c r="H12" s="27"/>
     </row>
     <row r="13" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="68"/>
+      <c r="F13" s="68"/>
+      <c r="G13" s="69"/>
       <c r="H13" s="27"/>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
+      <c r="F14" s="68"/>
+      <c r="G14" s="69"/>
       <c r="H14" s="27"/>
     </row>
     <row r="15" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="69"/>
       <c r="H15" s="27"/>
     </row>
     <row r="16" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
-      <c r="B16" s="54"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="54"/>
+      <c r="B16" s="67"/>
+      <c r="C16" s="68"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="69"/>
       <c r="H16" s="27"/>
     </row>
     <row r="17" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
-      <c r="B17" s="59" t="s">
-        <v>188</v>
-      </c>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
+      <c r="B17" s="70" t="s">
+        <v>181</v>
+      </c>
+      <c r="C17" s="71"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="72"/>
       <c r="H17" s="30"/>
     </row>
     <row r="18" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
-      <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="58"/>
-      <c r="F18" s="58"/>
-      <c r="G18" s="58"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
       <c r="H18" s="30"/>
     </row>
     <row r="19" spans="1:8" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19"/>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
       <c r="H19" s="30"/>
     </row>
   </sheetData>
@@ -2791,7 +2929,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
@@ -2819,7 +2957,7 @@
         <v>37</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2859,7 +2997,7 @@
         <v>39</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2879,7 +3017,7 @@
         <v>40</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2967,69 +3105,6 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>